<commit_message>
HW03 Started and Timed Lab 1
</commit_message>
<xml_diff>
--- a/hw03/kmap.xlsx
+++ b/hw03/kmap.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10514"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://gtvault-my.sharepoint.com/personal/zakkawi3_gatech_edu/Documents/Desktop/Georgia Tech/Spring 2023/CS 2110/hw03 revisions/HW-StateMachines/student/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huan\Documents\GT\Summer 2023\CS_2110\hw03\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="89" documentId="13_ncr:1_{FDC25BD4-D9F0-2743-8BED-F63FD615113D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1972D7FC-3C51-0149-A30B-0580BD68E69F}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D92302B-0F07-4585-8B52-0BF2849E122F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="14900" windowHeight="16180" xr2:uid="{E669F371-B88B-4909-8EAE-8F389B6E16B2}"/>
+    <workbookView xWindow="-90" yWindow="0" windowWidth="9250" windowHeight="13770" xr2:uid="{E669F371-B88B-4909-8EAE-8F389B6E16B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="20">
   <si>
     <t>S1'S0'</t>
   </si>
@@ -82,6 +82,18 @@
   </si>
   <si>
     <t>S</t>
+  </si>
+  <si>
+    <t>S1'S0' 00</t>
+  </si>
+  <si>
+    <t>S1'S0 01</t>
+  </si>
+  <si>
+    <t>S1S0 11</t>
+  </si>
+  <si>
+    <t>S1S0' 10</t>
   </si>
 </sst>
 </file>
@@ -164,10 +176,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -468,52 +476,68 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5F6CD62-9EA1-4796-8420-5C827DF2B464}">
   <dimension ref="A1:H19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="7" max="7" width="18.5" customWidth="1"/>
-    <col min="8" max="8" width="31.1640625" customWidth="1"/>
+    <col min="7" max="7" width="18.453125" customWidth="1"/>
+    <col min="8" max="8" width="31.1796875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="G1" s="2"/>
       <c r="H1" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B2" s="1"/>
-      <c r="C2" s="1"/>
-      <c r="D2" s="1"/>
-      <c r="E2" s="1"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B2" s="1">
+        <v>1</v>
+      </c>
+      <c r="C2" s="1">
+        <v>0</v>
+      </c>
+      <c r="D2" s="1">
+        <v>1</v>
+      </c>
+      <c r="E2" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B3" s="1"/>
-      <c r="C3" s="1"/>
-      <c r="D3" s="1"/>
-      <c r="E3" s="1"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B3" s="1">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1">
+        <v>1</v>
+      </c>
+      <c r="D3" s="1">
+        <v>1</v>
+      </c>
+      <c r="E3" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -534,25 +558,41 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B6" s="1"/>
-      <c r="C6" s="1"/>
-      <c r="D6" s="1"/>
-      <c r="E6" s="1"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B6" s="1">
+        <v>0</v>
+      </c>
+      <c r="C6" s="1">
+        <v>1</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B7" s="1"/>
-      <c r="C7" s="1"/>
-      <c r="D7" s="1"/>
-      <c r="E7" s="1"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B7" s="1">
+        <v>0</v>
+      </c>
+      <c r="C7" s="1">
+        <v>0</v>
+      </c>
+      <c r="D7" s="1">
+        <v>0</v>
+      </c>
+      <c r="E7" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -573,25 +613,41 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B10" s="1"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B10" s="1">
+        <v>1</v>
+      </c>
+      <c r="C10" s="1">
+        <v>1</v>
+      </c>
+      <c r="D10" s="1">
+        <v>0</v>
+      </c>
+      <c r="E10" s="1">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A11" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B11" s="1"/>
-      <c r="C11" s="1"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.2">
+      <c r="B11" s="1">
+        <v>1</v>
+      </c>
+      <c r="C11" s="1">
+        <v>1</v>
+      </c>
+      <c r="D11" s="1">
+        <v>0</v>
+      </c>
+      <c r="E11" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A13" s="1" t="s">
         <v>4</v>
       </c>
@@ -612,7 +668,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
@@ -621,7 +677,7 @@
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -630,7 +686,7 @@
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
         <v>6</v>
       </c>
@@ -651,7 +707,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A18" s="1" t="s">
         <v>13</v>
       </c>
@@ -660,7 +716,7 @@
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
     </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>14</v>
       </c>

</xml_diff>

<commit_message>
Finished excel table and Completed fsm
</commit_message>
<xml_diff>
--- a/hw03/kmap.xlsx
+++ b/hw03/kmap.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huan\Documents\GT\Summer 2023\CS_2110\hw03\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D92302B-0F07-4585-8B52-0BF2849E122F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C8DC68CE-E75F-4E2D-B081-D0F735507577}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="0" windowWidth="9250" windowHeight="13770" xr2:uid="{E669F371-B88B-4909-8EAE-8F389B6E16B2}"/>
+    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="13770" xr2:uid="{E669F371-B88B-4909-8EAE-8F389B6E16B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="50" uniqueCount="31">
   <si>
     <t>S1'S0'</t>
   </si>
@@ -94,6 +94,39 @@
   </si>
   <si>
     <t>S1S0' 10</t>
+  </si>
+  <si>
+    <t>G' 0</t>
+  </si>
+  <si>
+    <t>G  1</t>
+  </si>
+  <si>
+    <t>S1'S0+S1S0'</t>
+  </si>
+  <si>
+    <t>S0'+GS0S1'</t>
+  </si>
+  <si>
+    <t>G'S1'S0+G'S1S0'</t>
+  </si>
+  <si>
+    <t>Notably, this is</t>
+  </si>
+  <si>
+    <t>S1 ^ S0</t>
+  </si>
+  <si>
+    <t>xor</t>
+  </si>
+  <si>
+    <t>G'(S1'S0+S1S0')</t>
+  </si>
+  <si>
+    <t>G'(S1 ^ S0)</t>
+  </si>
+  <si>
+    <t>S1'+S0</t>
   </si>
 </sst>
 </file>
@@ -498,31 +531,33 @@
       <c r="E1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="G1" s="2"/>
+      <c r="G1" s="2" t="s">
+        <v>30</v>
+      </c>
       <c r="H1" s="3" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A2" s="1" t="s">
-        <v>13</v>
+        <v>20</v>
       </c>
       <c r="B2" s="1">
         <v>1</v>
       </c>
       <c r="C2" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D2" s="1">
         <v>1</v>
       </c>
       <c r="E2" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A3" s="1" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B3" s="1">
         <v>1</v>
@@ -534,7 +569,7 @@
         <v>1</v>
       </c>
       <c r="E3" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.35">
@@ -553,7 +588,9 @@
       <c r="E5" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G5" s="2"/>
+      <c r="G5" s="2" t="s">
+        <v>3</v>
+      </c>
       <c r="H5" s="3" t="s">
         <v>11</v>
       </c>
@@ -566,13 +603,13 @@
         <v>0</v>
       </c>
       <c r="C6" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D6" s="1">
         <v>0</v>
       </c>
       <c r="E6" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.35">
@@ -589,7 +626,7 @@
         <v>0</v>
       </c>
       <c r="E7" s="1">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.35">
@@ -608,7 +645,9 @@
       <c r="E9" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G9" s="2"/>
+      <c r="G9" s="2" t="s">
+        <v>22</v>
+      </c>
       <c r="H9" s="3" t="s">
         <v>12</v>
       </c>
@@ -618,7 +657,7 @@
         <v>13</v>
       </c>
       <c r="B10" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C10" s="1">
         <v>1</v>
@@ -627,7 +666,10 @@
         <v>0</v>
       </c>
       <c r="E10" s="1">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G10" t="s">
+        <v>25</v>
       </c>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.35">
@@ -635,7 +677,7 @@
         <v>14</v>
       </c>
       <c r="B11" s="1">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" s="1">
         <v>1</v>
@@ -645,6 +687,14 @@
       </c>
       <c r="E11" s="1">
         <v>1</v>
+      </c>
+      <c r="G11" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+      <c r="G12" t="s">
+        <v>27</v>
       </c>
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.35">
@@ -663,7 +713,9 @@
       <c r="E13" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G13" s="2"/>
+      <c r="G13" s="2" t="s">
+        <v>23</v>
+      </c>
       <c r="H13" s="3" t="s">
         <v>5</v>
       </c>
@@ -672,19 +724,35 @@
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B14" s="1"/>
-      <c r="C14" s="1"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
+      <c r="B14" s="1">
+        <v>1</v>
+      </c>
+      <c r="C14" s="1">
+        <v>0</v>
+      </c>
+      <c r="D14" s="1">
+        <v>0</v>
+      </c>
+      <c r="E14" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B15" s="1"/>
-      <c r="C15" s="1"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
+      <c r="B15" s="1">
+        <v>1</v>
+      </c>
+      <c r="C15" s="1">
+        <v>1</v>
+      </c>
+      <c r="D15" s="1">
+        <v>0</v>
+      </c>
+      <c r="E15" s="1">
+        <v>1</v>
+      </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A17" s="1" t="s">
@@ -702,7 +770,9 @@
       <c r="E17" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="G17" s="2"/>
+      <c r="G17" s="2" t="s">
+        <v>24</v>
+      </c>
       <c r="H17" s="3" t="s">
         <v>7</v>
       </c>
@@ -711,19 +781,41 @@
       <c r="A18" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="B18" s="1"/>
-      <c r="C18" s="1"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
+      <c r="B18" s="1">
+        <v>0</v>
+      </c>
+      <c r="C18" s="1">
+        <v>1</v>
+      </c>
+      <c r="D18" s="1">
+        <v>0</v>
+      </c>
+      <c r="E18" s="1">
+        <v>1</v>
+      </c>
+      <c r="G18" t="s">
+        <v>28</v>
+      </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.35">
       <c r="A19" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="B19" s="1"/>
-      <c r="C19" s="1"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
+      <c r="B19" s="1">
+        <v>0</v>
+      </c>
+      <c r="C19" s="1">
+        <v>0</v>
+      </c>
+      <c r="D19" s="1">
+        <v>0</v>
+      </c>
+      <c r="E19" s="1">
+        <v>0</v>
+      </c>
+      <c r="G19" t="s">
+        <v>29</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fixed a bit of hw03
</commit_message>
<xml_diff>
--- a/hw03/kmap.xlsx
+++ b/hw03/kmap.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="26327"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24332"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\huan\Documents\GT\Summer 2023\CS_2110\hw03\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bruh\Documents\GT\Summer 2023\CS_2110\hw03\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1A39C4FA-A2C6-492B-BCC7-78B37518317C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E59BAE8-B686-499D-B2CF-7593BB02F1FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="12710" yWindow="0" windowWidth="12980" windowHeight="13770" xr2:uid="{E669F371-B88B-4909-8EAE-8F389B6E16B2}"/>
+    <workbookView xWindow="-17376" yWindow="3744" windowWidth="17472" windowHeight="6312" xr2:uid="{E669F371-B88B-4909-8EAE-8F389B6E16B2}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -105,12 +105,6 @@
     <t>S1'S0+S1S0'</t>
   </si>
   <si>
-    <t>S0'+GS0S1'</t>
-  </si>
-  <si>
-    <t>G'S1'S0+G'S1S0'</t>
-  </si>
-  <si>
     <t>Notably, this is</t>
   </si>
   <si>
@@ -120,12 +114,6 @@
     <t>xor</t>
   </si>
   <si>
-    <t>G'(S1'S0+S1S0')</t>
-  </si>
-  <si>
-    <t>G'(S1 ^ S0)</t>
-  </si>
-  <si>
     <t>S1'+S0</t>
   </si>
   <si>
@@ -136,6 +124,18 @@
   </si>
   <si>
     <t>by De Morgan's</t>
+  </si>
+  <si>
+    <t>S0'+S0S1'G</t>
+  </si>
+  <si>
+    <t>S1'S0G'+S1S0'G'</t>
+  </si>
+  <si>
+    <t>(S1'S0+S1S0')G'</t>
+  </si>
+  <si>
+    <t>(S1 ^ S0)G'</t>
   </si>
 </sst>
 </file>
@@ -518,13 +518,13 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F5F6CD62-9EA1-4796-8420-5C827DF2B464}">
   <dimension ref="A1:H19"/>
-  <sheetFormatPr defaultColWidth="8.81640625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="7" max="7" width="18.453125" customWidth="1"/>
-    <col min="8" max="8" width="31.1796875" customWidth="1"/>
+    <col min="7" max="7" width="18.44140625" customWidth="1"/>
+    <col min="8" max="8" width="31.21875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>8</v>
       </c>
@@ -541,13 +541,13 @@
         <v>19</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="H1" s="3" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>20</v>
       </c>
@@ -564,10 +564,10 @@
         <v>0</v>
       </c>
       <c r="G2" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.35">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>21</v>
       </c>
@@ -584,15 +584,15 @@
         <v>0</v>
       </c>
       <c r="G3" t="s">
-        <v>32</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.35">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
       <c r="G4" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.35">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>9</v>
       </c>
@@ -615,7 +615,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>13</v>
       </c>
@@ -632,7 +632,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>14</v>
       </c>
@@ -649,7 +649,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>15</v>
       </c>
@@ -672,7 +672,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>13</v>
       </c>
@@ -689,10 +689,10 @@
         <v>1</v>
       </c>
       <c r="G10" t="s">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.35">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>14</v>
       </c>
@@ -709,15 +709,15 @@
         <v>1</v>
       </c>
       <c r="G11" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.35">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="G12" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.35">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>4</v>
       </c>
@@ -734,13 +734,13 @@
         <v>3</v>
       </c>
       <c r="G13" s="2" t="s">
-        <v>23</v>
+        <v>30</v>
       </c>
       <c r="H13" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>13</v>
       </c>
@@ -757,7 +757,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>14</v>
       </c>
@@ -774,7 +774,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>6</v>
       </c>
@@ -791,13 +791,13 @@
         <v>3</v>
       </c>
       <c r="G17" s="2" t="s">
-        <v>24</v>
+        <v>31</v>
       </c>
       <c r="H17" s="3" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>13</v>
       </c>
@@ -814,10 +814,10 @@
         <v>1</v>
       </c>
       <c r="G18" t="s">
-        <v>28</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.35">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>14</v>
       </c>
@@ -834,7 +834,7 @@
         <v>0</v>
       </c>
       <c r="G19" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>